<commit_message>
additional refactoring of files and documentation
</commit_message>
<xml_diff>
--- a/examples/example_player_rankings.xlsx
+++ b/examples/example_player_rankings.xlsx
@@ -2,18 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
-  <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3dbb7ad640958b53/Desktop/live draft board/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DB4542F1-A298-482F-AA79-815CF7710B07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <workbookPr filterPrivacy="1" defaultThemeVersion="202300"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{48D0799C-E354-4F2D-A956-CE111F34BA91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{D37C3534-F0C7-4860-AE65-1D2BAD9A18AC}"/>
   </bookViews>
   <sheets>
-    <sheet name="WWTS draft rankings" sheetId="1" r:id="rId1"/>
+    <sheet name="rankings" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>

</xml_diff>